<commit_message>
Update of the Mozambique shapefile to the new boundaries
</commit_message>
<xml_diff>
--- a/input_map/admin_levels.xlsx
+++ b/input_map/admin_levels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acted.sharepoint.com/sites/IMPACTHQ-PublicServices-IMPACT-Education/Documents partages/IMPACT - Education/Education - shared folder/PiN/PiN methodology studies 2025/new_dataset_testing/input_map/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\albertoramirez\Projects\pin-calculation-app\input_map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="8_{C2F32411-7B95-4D1A-BD4D-9D08D227516E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{478BD05E-E6D6-465C-967E-606DF069A70A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA75DF7-430A-4751-BD60-A7D855B7FC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{1A83F149-4476-49D1-A13F-AAA0E7368416}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{1A83F149-4476-49D1-A13F-AAA0E7368416}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="26">
   <si>
     <t>HNO2024</t>
   </si>
@@ -111,6 +111,12 @@
   </si>
   <si>
     <t>shapefile</t>
+  </si>
+  <si>
+    <t>LMR</t>
+  </si>
+  <si>
+    <t>MOZ</t>
   </si>
 </sst>
 </file>
@@ -520,18 +526,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{487AD388-BD61-48FE-9305-B931CF11F4A1}">
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" customWidth="1"/>
-    <col min="2" max="2" width="18.1328125" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" customWidth="1"/>
     <col min="3" max="4" width="15" customWidth="1"/>
-    <col min="5" max="6" width="12.1328125" customWidth="1"/>
-    <col min="7" max="7" width="13.5" customWidth="1"/>
-    <col min="8" max="8" width="12.1328125" customWidth="1"/>
+    <col min="5" max="6" width="12.109375" customWidth="1"/>
+    <col min="7" max="7" width="21.5546875" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" thickBot="1" x14ac:dyDescent="1.1499999999999999">
+    <row r="1" spans="1:8" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -557,7 +563,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.5" thickTop="1" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -579,8 +585,11 @@
       <c r="G2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -602,8 +611,11 @@
       <c r="G3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -625,8 +637,11 @@
       <c r="G4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -648,8 +663,11 @@
       <c r="G5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="H5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -671,8 +689,11 @@
       <c r="G6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="H6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -694,8 +715,11 @@
       <c r="G7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="H7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -709,137 +733,196 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.75">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.75">
-      <c r="A11" t="s">
+      <c r="H11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>22</v>
       </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.75">
-      <c r="A12" t="s">
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>16</v>
       </c>
-      <c r="B12" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.75">
-      <c r="A13" t="s">
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>17</v>
       </c>
-      <c r="B13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.75">
-      <c r="A14" t="s">
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>18</v>
       </c>
-      <c r="D14" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" t="s">
-        <v>19</v>
+      <c r="D16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{487AD388-BD61-48FE-9305-B931CF11F4A1}"/>
+  <autoFilter ref="A1:H1" xr:uid="{487AD388-BD61-48FE-9305-B931CF11F4A1}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H16">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1098,7 +1181,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC48FFD0-0D2D-4174-9E5B-CAFB09488FCD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC48FFD0-0D2D-4174-9E5B-CAFB09488FCD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
+    <ds:schemaRef ds:uri="14cbb838-50ff-4dab-9c3f-cddf75f03c13"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Update the admin file with Sparkea
</commit_message>
<xml_diff>
--- a/input_map/admin_levels.xlsx
+++ b/input_map/admin_levels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\albertoramirez\Projects\pin-calculation-app\input_map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA75DF7-430A-4751-BD60-A7D855B7FC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877968AA-75D6-481C-8A50-6095C83B6F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{1A83F149-4476-49D1-A13F-AAA0E7368416}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="27">
   <si>
     <t>HNO2024</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>MOZ</t>
+  </si>
+  <si>
+    <t>SPA</t>
   </si>
 </sst>
 </file>
@@ -526,7 +529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{487AD388-BD61-48FE-9305-B931CF11F4A1}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.5546875" customWidth="1"/>
@@ -917,6 +920,14 @@
         <v>20</v>
       </c>
     </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{487AD388-BD61-48FE-9305-B931CF11F4A1}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H16">
@@ -929,13 +940,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1162,20 +1172,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC78E818-E8A5-463C-A2DF-4621D8D99EFD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BD5855A-F4D0-4374-82E1-C9EDA19F7215}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1200,9 +1209,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BD5855A-F4D0-4374-82E1-C9EDA19F7215}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC78E818-E8A5-463C-A2DF-4621D8D99EFD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update with the right Pcode for Sparkea
</commit_message>
<xml_diff>
--- a/input_map/admin_levels.xlsx
+++ b/input_map/admin_levels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\albertoramirez\Projects\pin-calculation-app\input_map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877968AA-75D6-481C-8A50-6095C83B6F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13EA5547-728C-48D2-963B-F6D275B932C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{1A83F149-4476-49D1-A13F-AAA0E7368416}"/>
   </bookViews>
@@ -119,7 +119,7 @@
     <t>MOZ</t>
   </si>
   <si>
-    <t>SPA</t>
+    <t>SPR</t>
   </si>
 </sst>
 </file>
@@ -940,12 +940,13 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1172,19 +1173,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BD5855A-F4D0-4374-82E1-C9EDA19F7215}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC78E818-E8A5-463C-A2DF-4621D8D99EFD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1209,11 +1211,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC78E818-E8A5-463C-A2DF-4621D8D99EFD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BD5855A-F4D0-4374-82E1-C9EDA19F7215}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>